<commit_message>
updated resistor values for cipher box V2, added CH32 reinit on error detection, added averaging ADC over some parametr value
</commit_message>
<xml_diff>
--- a/projects/cipher_box/резисторы.xlsx
+++ b/projects/cipher_box/резисторы.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
   <si>
     <t>номиналы</t>
   </si>
@@ -46,6 +46,24 @@
   </si>
   <si>
     <t>Integral</t>
+  </si>
+  <si>
+    <t>4700|2200</t>
+  </si>
+  <si>
+    <t>5100|5100</t>
+  </si>
+  <si>
+    <t>6800|10000</t>
+  </si>
+  <si>
+    <t>6800|47000</t>
+  </si>
+  <si>
+    <t>10000|47000</t>
+  </si>
+  <si>
+    <t>20000|51000</t>
   </si>
 </sst>
 </file>
@@ -2278,10 +2296,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2316,7 +2334,7 @@
         <v>3300</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>0</v>
       </c>
@@ -2354,7 +2372,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>10</v>
       </c>
@@ -2392,7 +2410,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>22</v>
       </c>
@@ -2428,7 +2446,7 @@
         <v>48.761904761904759</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>47</v>
       </c>
@@ -2460,7 +2478,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>150</v>
       </c>
@@ -2496,7 +2514,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>200</v>
       </c>
@@ -2527,8 +2545,14 @@
         <f t="shared" si="5"/>
         <v>79</v>
       </c>
+      <c r="L7">
+        <v>20000</v>
+      </c>
+      <c r="M7">
+        <v>51000</v>
+      </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>270</v>
       </c>
@@ -2560,8 +2584,21 @@
         <f t="shared" si="5"/>
         <v>65</v>
       </c>
+      <c r="K8" t="s">
+        <v>9</v>
+      </c>
+      <c r="L8">
+        <f>(L7*M7)/(L7+M7)</f>
+        <v>14366.197183098591</v>
+      </c>
+      <c r="M8">
+        <v>15000</v>
+      </c>
+      <c r="N8">
+        <v>68000</v>
+      </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>330</v>
       </c>
@@ -2594,10 +2631,14 @@
       </c>
       <c r="J9">
         <f t="shared" si="5"/>
-        <v>68</v>
+        <v>58</v>
+      </c>
+      <c r="L9">
+        <f>-(M8*N8)/(M8-N8)</f>
+        <v>19245.283018867925</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>470</v>
       </c>
@@ -2614,23 +2655,25 @@
         <v>9</v>
       </c>
       <c r="G10" s="2">
-        <f>(G11+G9)/2</f>
-        <v>2650</v>
+        <v>2550</v>
       </c>
       <c r="H10" s="5">
         <f t="shared" si="3"/>
-        <v>1.808970099667774</v>
+        <v>1.8395270270270268</v>
       </c>
       <c r="I10">
         <f t="shared" si="4"/>
-        <v>561</v>
+        <v>571</v>
       </c>
       <c r="J10">
         <f t="shared" si="5"/>
-        <v>54</v>
+        <v>64</v>
+      </c>
+      <c r="K10" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>510</v>
       </c>
@@ -2663,10 +2706,10 @@
       </c>
       <c r="J11">
         <f t="shared" si="5"/>
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>680</v>
       </c>
@@ -2683,23 +2726,25 @@
         <v>61</v>
       </c>
       <c r="G12" s="2">
-        <f>(G13+G11)/2</f>
-        <v>4000</v>
+        <v>4047</v>
       </c>
       <c r="H12" s="5">
         <f t="shared" si="3"/>
-        <v>1.4776119402985073</v>
+        <v>1.4682486180396386</v>
       </c>
       <c r="I12">
         <f t="shared" si="4"/>
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="J12">
         <f t="shared" si="5"/>
-        <v>40</v>
+        <v>37</v>
+      </c>
+      <c r="K12" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>1000</v>
       </c>
@@ -2728,10 +2773,10 @@
       </c>
       <c r="J13">
         <f t="shared" si="5"/>
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>2000</v>
       </c>
@@ -2748,23 +2793,25 @@
         <v>22</v>
       </c>
       <c r="G14" s="2">
-        <f>(G15+G13)/2</f>
-        <v>5750</v>
+        <v>5940</v>
       </c>
       <c r="H14" s="5">
         <f t="shared" si="3"/>
-        <v>1.1940789473684208</v>
+        <v>1.1697099892588612</v>
       </c>
       <c r="I14">
         <f t="shared" si="4"/>
-        <v>371</v>
+        <v>363</v>
       </c>
       <c r="J14">
         <f t="shared" si="5"/>
-        <v>39</v>
+        <v>31</v>
+      </c>
+      <c r="K14" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>2200</v>
       </c>
@@ -2793,10 +2840,10 @@
       </c>
       <c r="J15">
         <f t="shared" si="5"/>
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>3300</v>
       </c>
@@ -2817,23 +2864,25 @@
         <v>122</v>
       </c>
       <c r="G16" s="2">
-        <f>(G17+G15)/2</f>
-        <v>8400</v>
+        <v>8245</v>
       </c>
       <c r="H16" s="5">
         <f t="shared" si="3"/>
-        <v>0.92523364485981308</v>
+        <v>0.93758071459319847</v>
       </c>
       <c r="I16">
         <f t="shared" si="4"/>
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="J16">
         <f t="shared" si="5"/>
-        <v>34</v>
+        <v>38</v>
+      </c>
+      <c r="K16" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>4700</v>
       </c>
@@ -2862,10 +2911,10 @@
       </c>
       <c r="J17">
         <f t="shared" si="5"/>
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>5100</v>
       </c>
@@ -2882,23 +2931,25 @@
         <v>67</v>
       </c>
       <c r="G18" s="2">
-        <f>(G19+G17)/2</f>
-        <v>15000</v>
+        <v>14366</v>
       </c>
       <c r="H18" s="5">
         <f t="shared" si="3"/>
-        <v>0.59281437125748493</v>
+        <v>0.61400541271989173</v>
       </c>
       <c r="I18">
         <f t="shared" si="4"/>
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="J18">
         <f t="shared" si="5"/>
-        <v>39</v>
+        <v>46</v>
+      </c>
+      <c r="K18" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>6800</v>
       </c>
@@ -2934,7 +2985,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>10000</v>
       </c>
@@ -2966,7 +3017,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>20000</v>
       </c>
@@ -2998,7 +3049,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>47000</v>
       </c>
@@ -3015,7 +3066,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>51000</v>
       </c>
@@ -3032,7 +3083,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>68000</v>
       </c>
@@ -3049,7 +3100,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>100000</v>
       </c>
@@ -3070,7 +3121,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>220000</v>
       </c>
@@ -3087,7 +3138,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>300000</v>
       </c>
@@ -3104,7 +3155,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>470000</v>
       </c>
@@ -3121,7 +3172,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>680000</v>
       </c>
@@ -3138,7 +3189,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>1000000</v>
       </c>

</xml_diff>